<commit_message>
Give the BOM's plates and printed parts their materials
The Source column now says how each was made: Ponoko laser cutting in
6.7 mm amber bamboo plywood, and Xometry 3D printing in white Nylon 12
(the parts were printed, not machined).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cad/scanner_mount_bom.xlsx
+++ b/cad/scanner_mount_bom.xlsx
@@ -244,7 +244,7 @@
     <t xml:space="preserve">374 x 352 x 6.7 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Laser cut (Ponoko DXF)</t>
+    <t xml:space="preserve">Ponoko - 6.7mm Amber Bamboo Plywood - Laser Cutting</t>
   </si>
   <si>
     <t xml:space="preserve">Lat/lon plate</t>
@@ -259,7 +259,7 @@
     <t xml:space="preserve">268 x 228 x 6.7 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">3D printed / machined parts</t>
+    <t xml:space="preserve">3D printed parts</t>
   </si>
   <si>
     <t xml:space="preserve">Printed part</t>
@@ -271,7 +271,7 @@
     <t xml:space="preserve">22.5 x 14.9 x 14.7 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">3D print / machined (Xometry STL)</t>
+    <t xml:space="preserve">Xometry - Nylon 12, White, Color: As Printed, Off White (Natural)</t>
   </si>
   <si>
     <t xml:space="preserve">Latitude stepper mount</t>
@@ -1499,7 +1499,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Add the control board's 24 V power supply to the BOM
A 24 V, 6 A AC adapter (100-240 V AC in, 5.5 x 2.1 mm jack with a
terminal connector) from Amazon, added by hand like the motor cables: a
counted row in the Wiring group on By sub-assembly, a row under the
purchased electronics on the Full BOM, and a Notes entry quoting the
listing title. The SUMIFS ranges over By sub-assembly grew by the one
row; the totals went from 112 to 113 part instances and the McMaster
order is unchanged. Recalculated in LibreOffice, no formula errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cad/scanner_mount_bom.xlsx
+++ b/cad/scanner_mount_bom.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="215">
   <si>
     <t xml:space="preserve">Revopoint scanner mount - McMaster-Carr order list</t>
   </si>
@@ -364,6 +364,18 @@
     <t xml:space="preserve">Amazon, sold in 3-packs (one pack covers both motors)</t>
   </si>
   <si>
+    <t xml:space="preserve">Power supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 V DC power supply for the control board</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 A, 100-240 V AC in, 5.5 x 2.1 mm jack with terminal connector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon</t>
+  </si>
+  <si>
     <t xml:space="preserve">Reference geometry (not purchased)</t>
   </si>
   <si>
@@ -442,16 +454,16 @@
     <t xml:space="preserve">    in the assembly, so its thread could not be confirmed from the geometry - confirm it against the McMaster listing.</t>
   </si>
   <si>
-    <t xml:space="preserve">  - Apart from the motor cables added below, the BOM has no wiring, belts, connectors or fasteners for the SKR Mini E3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    board beyond the four M3 standoff kits, and no fasteners holding the Revopoint scanner to the scanner mount plate.</t>
+    <t xml:space="preserve">  - Apart from the motor cables and power supply added below, the BOM has no wiring, belts, connectors or fasteners for the</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    SKR Mini E3 board beyond the four M3 standoff kits, and no fasteners holding the Revopoint scanner to the scanner mount plate.</t>
   </si>
   <si>
     <t xml:space="preserve">  - The Revopoint scanner parts and the "small_head" test object are reference geometry, not items to buy.</t>
   </si>
   <si>
-    <t xml:space="preserve">Added by hand on 27 Oct 2026, not counted from the model:</t>
+    <t xml:space="preserve">Added by hand on 27 and 28 Oct 2026, not counted from the model:</t>
   </si>
   <si>
     <t xml:space="preserve">  - Counterweights: two ~1.25" (32 mm) pieces of 1/2" x 1/2" copper bar (McMaster-Carr 89275K36, 6" long), one held</t>
@@ -475,6 +487,15 @@
     <t xml:space="preserve">    ("3Pcs 1.5M Stepper Motor Cables XH2.54 4Pin to 6Pin Terminal Motor Wires ..."). One pack covers both motors.</t>
   </si>
   <si>
+    <t xml:space="preserve">  - Power supply (28 Oct): one 24 V, 6 A AC adapter (100-240 V AC in) for the SKR Mini E3 board, from Amazon:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    "24V Power Supply, 24 Volt 6 Amp AC DC Adapter 100V-240V AC to 24V DC Power Supply with LED Terminal Connector,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    5A 4A 3A 2A 1A DC Adapter with 5.5x2.1mm Jack".</t>
+  </si>
+  <si>
     <t xml:space="preserve">  - counter_weight.FCStd (exported to Xometry on 10 Oct) was an earlier counterweight design and is not part of the build.</t>
   </si>
   <si>
@@ -635,6 +656,9 @@
   </si>
   <si>
     <t xml:space="preserve">Stepper motor cable, XH2.54 4-pin to 6-pin - 1.5 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 V DC power supply for the control board - 6 A, 100-240 V AC in, 5.5 x 2.1 mm jack with terminal connector</t>
   </si>
   <si>
     <t xml:space="preserve">Revopoint scanner (reference)</t>
@@ -1145,7 +1169,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B6)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B6)</f>
         <v>4</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -1166,7 +1190,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B7)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B7)</f>
         <v>16</v>
       </c>
       <c r="B7" s="8" t="s">
@@ -1187,7 +1211,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B8)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B8)</f>
         <v>2</v>
       </c>
       <c r="B8" s="8" t="s">
@@ -1208,7 +1232,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B9)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B9)</f>
         <v>12</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -1229,7 +1253,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B10)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B10)</f>
         <v>10</v>
       </c>
       <c r="B10" s="8" t="s">
@@ -1250,7 +1274,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B11)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B11)</f>
         <v>12</v>
       </c>
       <c r="B11" s="8" t="s">
@@ -1281,7 +1305,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B14)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B14)</f>
         <v>12</v>
       </c>
       <c r="B14" s="8" t="s">
@@ -1312,7 +1336,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B17)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B17)</f>
         <v>4</v>
       </c>
       <c r="B17" s="8" t="s">
@@ -1333,7 +1357,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B18)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B18)</f>
         <v>8</v>
       </c>
       <c r="B18" s="8" t="s">
@@ -1354,7 +1378,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B19)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B19)</f>
         <v>4</v>
       </c>
       <c r="B19" s="8" t="s">
@@ -1385,7 +1409,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B22)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B22)</f>
         <v>4</v>
       </c>
       <c r="B22" s="8" t="s">
@@ -1416,7 +1440,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$D$2:$D$39,$B25)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B25)</f>
         <v>1</v>
       </c>
       <c r="B25" s="8" t="s">
@@ -1491,7 +1515,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -1801,7 +1825,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D19&amp;IF($E19="-",""," - "&amp;$E19))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D19&amp;IF($E19="-",""," - "&amp;$E19))</f>
         <v>1</v>
       </c>
       <c r="B19" s="8"/>
@@ -1820,7 +1844,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D20&amp;IF($E20="-",""," - "&amp;$E20))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D20&amp;IF($E20="-",""," - "&amp;$E20))</f>
         <v>1</v>
       </c>
       <c r="B20" s="8"/>
@@ -1839,7 +1863,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D21&amp;IF($E21="-",""," - "&amp;$E21))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D21&amp;IF($E21="-",""," - "&amp;$E21))</f>
         <v>1</v>
       </c>
       <c r="B21" s="8"/>
@@ -1868,7 +1892,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D24&amp;IF($E24="-",""," - "&amp;$E24))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D24&amp;IF($E24="-",""," - "&amp;$E24))</f>
         <v>2</v>
       </c>
       <c r="B24" s="8"/>
@@ -1887,7 +1911,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D25&amp;IF($E25="-",""," - "&amp;$E25))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D25&amp;IF($E25="-",""," - "&amp;$E25))</f>
         <v>2</v>
       </c>
       <c r="B25" s="8"/>
@@ -1906,7 +1930,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D26&amp;IF($E26="-",""," - "&amp;$E26))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D26&amp;IF($E26="-",""," - "&amp;$E26))</f>
         <v>1</v>
       </c>
       <c r="B26" s="8"/>
@@ -1925,7 +1949,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D27&amp;IF($E27="-",""," - "&amp;$E27))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D27&amp;IF($E27="-",""," - "&amp;$E27))</f>
         <v>1</v>
       </c>
       <c r="B27" s="8"/>
@@ -1944,7 +1968,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D28&amp;IF($E28="-",""," - "&amp;$E28))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D28&amp;IF($E28="-",""," - "&amp;$E28))</f>
         <v>1</v>
       </c>
       <c r="B28" s="8"/>
@@ -1963,7 +1987,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D29&amp;IF($E29="-",""," - "&amp;$E29))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D29&amp;IF($E29="-",""," - "&amp;$E29))</f>
         <v>1</v>
       </c>
       <c r="B29" s="8"/>
@@ -1992,7 +2016,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D32&amp;IF($E32="-",""," - "&amp;$E32))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D32&amp;IF($E32="-",""," - "&amp;$E32))</f>
         <v>2</v>
       </c>
       <c r="B32" s="8"/>
@@ -2021,7 +2045,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D35&amp;IF($E35="-",""," - "&amp;$E35))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D35&amp;IF($E35="-",""," - "&amp;$E35))</f>
         <v>1</v>
       </c>
       <c r="B35" s="8"/>
@@ -2040,7 +2064,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D36&amp;IF($E36="-",""," - "&amp;$E36))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D36&amp;IF($E36="-",""," - "&amp;$E36))</f>
         <v>1</v>
       </c>
       <c r="B36" s="8"/>
@@ -2059,7 +2083,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D37&amp;IF($E37="-",""," - "&amp;$E37))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D37&amp;IF($E37="-",""," - "&amp;$E37))</f>
         <v>1</v>
       </c>
       <c r="B37" s="8"/>
@@ -2078,7 +2102,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D38&amp;IF($E38="-",""," - "&amp;$E38))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D38&amp;IF($E38="-",""," - "&amp;$E38))</f>
         <v>2</v>
       </c>
       <c r="B38" s="8"/>
@@ -2095,118 +2119,137 @@
         <v>112</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D39&amp;IF($E39="-",""," - "&amp;$E39))</f>
+        <v>1</v>
+      </c>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="B40" s="6"/>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
+      <c r="D39" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F39" s="8" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D41&amp;IF($E41="-",""," - "&amp;$E41))</f>
-        <v>1</v>
-      </c>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="F41" s="8" t="s">
+      <c r="A41" s="5" t="s">
         <v>117</v>
       </c>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D42&amp;IF($E42="-",""," - "&amp;$E42))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D42&amp;IF($E42="-",""," - "&amp;$E42))</f>
         <v>1</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="8" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D43&amp;IF($E43="-",""," - "&amp;$E43))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D43&amp;IF($E43="-",""," - "&amp;$E43))</f>
         <v>1</v>
       </c>
       <c r="B43" s="8"/>
       <c r="C43" s="8" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D44&amp;IF($E44="-",""," - "&amp;$E44))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D44&amp;IF($E44="-",""," - "&amp;$E44))</f>
         <v>1</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="8" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D44" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E44" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="E44" s="8" t="s">
-        <v>116</v>
-      </c>
       <c r="F44" s="8" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$39,'By sub-assembly'!$E$2:$E$39,$D45&amp;IF($E45="-",""," - "&amp;$E45))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D45&amp;IF($E45="-",""," - "&amp;$E45))</f>
         <v>1</v>
       </c>
       <c r="B45" s="8"/>
       <c r="C45" s="8" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D45" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F45" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="E45" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="10" t="n">
-        <f aca="false">SUM(A4:A46)</f>
-        <v>112</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>123</v>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D46&amp;IF($E46="-",""," - "&amp;$E46))</f>
+        <v>1</v>
+      </c>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="10" t="n">
+        <f aca="false">SUM(A4:A47)</f>
+        <v>113</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -2225,7 +2268,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="125"/>
@@ -2233,7 +2276,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2241,17 +2284,17 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2259,42 +2302,42 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2302,32 +2345,32 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2335,60 +2378,75 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12"/>
+      <c r="A32" s="12" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>152</v>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="12"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="12" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -2407,7 +2465,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
@@ -2420,13 +2478,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>65</v>
@@ -2435,10 +2493,10 @@
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2446,7 +2504,7 @@
         <v>56</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1</v>
@@ -2455,7 +2513,7 @@
         <v>52</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="F2" s="13" t="n">
         <v>1</v>
@@ -2470,14 +2528,14 @@
         <v>56</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="F3" s="13" t="n">
         <v>1</v>
@@ -2492,14 +2550,14 @@
         <v>56</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="F4" s="13" t="n">
         <v>1</v>
@@ -2511,17 +2569,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="F5" s="13" t="n">
         <v>1</v>
@@ -2533,17 +2591,17 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="8"/>
       <c r="E6" s="8" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="F6" s="13" t="n">
         <v>1</v>
@@ -2558,7 +2616,7 @@
         <v>50</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>4</v>
@@ -2567,7 +2625,7 @@
         <v>46</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="F7" s="13" t="n">
         <v>1</v>
@@ -2582,7 +2640,7 @@
         <v>50</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>4</v>
@@ -2591,7 +2649,7 @@
         <v>25</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="F8" s="13" t="n">
         <v>1</v>
@@ -2606,7 +2664,7 @@
         <v>13</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>4</v>
@@ -2615,7 +2673,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="F9" s="13" t="n">
         <v>1</v>
@@ -2630,7 +2688,7 @@
         <v>13</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>4</v>
@@ -2639,7 +2697,7 @@
         <v>20</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="F10" s="13" t="n">
         <v>1</v>
@@ -2654,7 +2712,7 @@
         <v>13</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>4</v>
@@ -2663,7 +2721,7 @@
         <v>35</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="F11" s="13" t="n">
         <v>1</v>
@@ -2678,7 +2736,7 @@
         <v>44</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>4</v>
@@ -2687,7 +2745,7 @@
         <v>25</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="F12" s="13" t="n">
         <v>2</v>
@@ -2702,7 +2760,7 @@
         <v>44</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>4</v>
@@ -2711,7 +2769,7 @@
         <v>42</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="F13" s="13" t="n">
         <v>1</v>
@@ -2723,17 +2781,17 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>1</v>
@@ -2748,7 +2806,7 @@
         <v>41</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>8</v>
@@ -2757,7 +2815,7 @@
         <v>14</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="F15" s="13" t="n">
         <v>1</v>
@@ -2772,7 +2830,7 @@
         <v>41</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>8</v>
@@ -2781,7 +2839,7 @@
         <v>20</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>1</v>
@@ -2796,7 +2854,7 @@
         <v>41</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>8</v>
@@ -2805,7 +2863,7 @@
         <v>39</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="F17" s="13" t="n">
         <v>1</v>
@@ -2817,17 +2875,17 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="F18" s="13" t="n">
         <v>1</v>
@@ -2839,10 +2897,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1</v>
@@ -2851,7 +2909,7 @@
         <v>14</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="F19" s="13" t="n">
         <v>4</v>
@@ -2863,10 +2921,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1</v>
@@ -2875,7 +2933,7 @@
         <v>30</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="F20" s="13" t="n">
         <v>7</v>
@@ -2887,17 +2945,17 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="8" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="F21" s="13" t="n">
         <v>1</v>
@@ -2909,17 +2967,17 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="F22" s="13" t="n">
         <v>2</v>
@@ -2931,17 +2989,17 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="F23" s="13" t="n">
         <v>1</v>
@@ -2953,17 +3011,17 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="F24" s="13" t="n">
         <v>1</v>
@@ -2975,17 +3033,17 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="F25" s="13" t="n">
         <v>2</v>
@@ -2997,10 +3055,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1</v>
@@ -3009,7 +3067,7 @@
         <v>17</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="F26" s="13" t="n">
         <v>1</v>
@@ -3021,10 +3079,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1</v>
@@ -3033,7 +3091,7 @@
         <v>23</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="F27" s="13" t="n">
         <v>6</v>
@@ -3045,10 +3103,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1</v>
@@ -3057,7 +3115,7 @@
         <v>30</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="F28" s="13" t="n">
         <v>5</v>
@@ -3069,17 +3127,17 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="F29" s="13" t="n">
         <v>1</v>
@@ -3091,17 +3149,17 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="F30" s="13" t="n">
         <v>1</v>
@@ -3113,10 +3171,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1</v>
@@ -3125,7 +3183,7 @@
         <v>17</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="F31" s="13" t="n">
         <v>1</v>
@@ -3137,10 +3195,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1</v>
@@ -3149,7 +3207,7 @@
         <v>23</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="F32" s="13" t="n">
         <v>4</v>
@@ -3161,17 +3219,17 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D33" s="8"/>
       <c r="E33" s="8" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="F33" s="13" t="n">
         <v>1</v>
@@ -3183,10 +3241,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1</v>
@@ -3195,7 +3253,7 @@
         <v>14</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="F34" s="13" t="n">
         <v>4</v>
@@ -3207,17 +3265,17 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="F35" s="13" t="n">
         <v>2</v>
@@ -3229,17 +3287,17 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8" t="s">
-        <v>115</v>
+        <v>211</v>
       </c>
       <c r="F36" s="13" t="n">
         <v>1</v>
@@ -3251,17 +3309,17 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D37" s="8"/>
       <c r="E37" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F37" s="13" t="n">
         <v>1</v>
@@ -3273,17 +3331,17 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="8" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="8"/>
       <c r="E38" s="8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F38" s="13" t="n">
         <v>1</v>
@@ -3295,17 +3353,17 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F39" s="13" t="n">
         <v>1</v>
@@ -3316,12 +3374,34 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F40" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="G40" s="10" t="n">
-        <f aca="false">SUM(G2:G39)</f>
-        <v>112</v>
+      <c r="A40" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="C40" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="8" t="n">
+        <f aca="false">C40*F40</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F41" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="G41" s="10" t="n">
+        <f aca="false">SUM(G2:G40)</f>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add the scanner's mounting washers to the BOM
Two McMaster-Carr 96659A106 18-8 stainless SAE washers (1/4" screw size,
0.281" ID, 0.625" OD) hold the scanner on its mount. The model doesn't
show them, so they are a hand-added row at the top level, with a Washers
section on the McMaster order and a row in the Full BOM.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cad/scanner_mount_bom.xlsx
+++ b/cad/scanner_mount_bom.xlsx
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="224">
   <si>
     <t xml:space="preserve">Revopoint scanner mount - McMaster-Carr order list</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantities are for one complete build, counted from every instance in assembly.FCStd (model saved 11 Oct 2026). The copper bar is added by hand (see Notes).</t>
+    <t xml:space="preserve">Quantities are for one complete build, counted from every instance in assembly.FCStd (model saved 11 Oct 2026). The copper bar and the washers are added by hand (see Notes).</t>
   </si>
   <si>
     <t xml:space="preserve">Qty</t>
@@ -127,6 +127,24 @@
     <t xml:space="preserve">M3 x 0.5 mm, 5.5 mm wide, 2.4 mm thick</t>
   </si>
   <si>
+    <t xml:space="preserve">Washers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">96659A106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Washer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18-8 stainless SAE washer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/4" screw size, 0.281" ID, 0.625" OD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scanner mount (not modeled)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Standoffs</t>
   </si>
   <si>
@@ -454,16 +472,16 @@
     <t xml:space="preserve">    in the assembly, so its thread could not be confirmed from the geometry - confirm it against the McMaster listing.</t>
   </si>
   <si>
-    <t xml:space="preserve">  - Apart from the motor cables and power supply added below, the BOM has no wiring, belts, connectors or fasteners for the</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    SKR Mini E3 board beyond the four M3 standoff kits, and no fasteners holding the Revopoint scanner to the scanner mount plate.</t>
+    <t xml:space="preserve">  - Apart from the motor cables, power supply and washers added below, the BOM has no wiring, belts, connectors or</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    fasteners for the SKR Mini E3 board beyond the four M3 standoff kits.</t>
   </si>
   <si>
     <t xml:space="preserve">  - The Revopoint scanner parts and the "small_head" test object are reference geometry, not items to buy.</t>
   </si>
   <si>
-    <t xml:space="preserve">Added by hand on 27 and 28 Oct 2026, not counted from the model:</t>
+    <t xml:space="preserve">Added by hand on 27, 28 and 29 Oct 2026, not counted from the model:</t>
   </si>
   <si>
     <t xml:space="preserve">  - Counterweights: two ~1.25" (32 mm) pieces of 1/2" x 1/2" copper bar (McMaster-Carr 89275K36, 6" long), one held</t>
@@ -496,6 +514,12 @@
     <t xml:space="preserve">    5A 4A 3A 2A 1A DC Adapter with 5.5x2.1mm Jack".</t>
   </si>
   <si>
+    <t xml:space="preserve">  - Washers (29 Oct): two 18-8 stainless SAE washers for 1/4" screws (0.281" ID, 0.625" OD), McMaster-Carr 96659A106,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    used in mounting the scanner. The model doesn't show them.</t>
+  </si>
+  <si>
     <t xml:space="preserve">  - counter_weight.FCStd (exported to Xometry on 10 Oct) was an earlier counterweight design and is not part of the build.</t>
   </si>
   <si>
@@ -529,6 +553,12 @@
     <t xml:space="preserve">Scanner mount plate - 268 x 228 x 6.7 mm</t>
   </si>
   <si>
+    <t xml:space="preserve">(not modeled)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18-8 stainless SAE washer - 1/4" screw size, 0.281" ID, 0.625" OD</t>
+  </si>
+  <si>
     <t xml:space="preserve">Scan test object (small bust) - 34.3 x 32.5 x 65.0 mm</t>
   </si>
   <si>
@@ -617,9 +647,6 @@
   </si>
   <si>
     <t xml:space="preserve">Latitude stepper arm - 38.0 x 40 x 16 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(not modeled)</t>
   </si>
   <si>
     <t xml:space="preserve">Counterweight, cut from copper bar - 1/2" x 1/2" x about 1.25" (32 mm) long</t>
@@ -1116,7 +1143,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -1169,7 +1196,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B6)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B6)</f>
         <v>4</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -1190,7 +1217,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B7)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B7)</f>
         <v>16</v>
       </c>
       <c r="B7" s="8" t="s">
@@ -1211,7 +1238,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B8)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B8)</f>
         <v>2</v>
       </c>
       <c r="B8" s="8" t="s">
@@ -1232,7 +1259,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B9)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B9)</f>
         <v>12</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -1253,7 +1280,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B10)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B10)</f>
         <v>10</v>
       </c>
       <c r="B10" s="8" t="s">
@@ -1274,7 +1301,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B11)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B11)</f>
         <v>12</v>
       </c>
       <c r="B11" s="8" t="s">
@@ -1305,7 +1332,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B14)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B14)</f>
         <v>12</v>
       </c>
       <c r="B14" s="8" t="s">
@@ -1336,8 +1363,8 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B17)</f>
-        <v>4</v>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B17)</f>
+        <v>2</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>35</v>
@@ -1352,74 +1379,74 @@
         <v>38</v>
       </c>
       <c r="F17" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B20)</f>
+        <v>4</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F20" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B18)</f>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B21)</f>
         <v>8</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B19)</f>
-        <v>4</v>
-      </c>
-      <c r="B19" s="8" t="s">
+      <c r="B21" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="8" t="s">
+      <c r="D21" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F19" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
+      <c r="E21" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B22)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B22)</f>
         <v>4</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>49</v>
@@ -1440,8 +1467,8 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$D$2:$D$40,$B25)</f>
-        <v>1</v>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B25)</f>
+        <v>4</v>
       </c>
       <c r="B25" s="8" t="s">
         <v>52</v>
@@ -1471,7 +1498,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="n">
-        <f aca="false">ROUNDUP('Full BOM'!A32*1.25/6,0)</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$D$2:$D$41,$B28)</f>
         <v>1</v>
       </c>
       <c r="B28" s="8" t="s">
@@ -1491,12 +1518,43 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="n">
-        <f aca="false">SUM(A6:A29)</f>
-        <v>90</v>
-      </c>
-      <c r="D30" s="10" t="s">
+      <c r="A30" s="5" t="s">
         <v>63</v>
+      </c>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="n">
+        <f aca="false">ROUNDUP('Full BOM'!A33*1.25/6,0)</f>
+        <v>1</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="n">
+        <f aca="false">SUM(A6:A32)</f>
+        <v>92</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1515,7 +1573,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -1528,7 +1586,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1536,7 +1594,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C3" s="11" t="s">
         <v>4</v>
@@ -1548,12 +1606,12 @@
         <v>6</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1563,44 +1621,44 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="n">
-        <f aca="false">'McMaster order'!A22</f>
+        <f aca="false">'McMaster order'!A25</f>
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
-        <f aca="false">'McMaster order'!A25</f>
+        <f aca="false">'McMaster order'!A28</f>
         <v>1</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1621,7 +1679,7 @@
         <v>33</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1642,7 +1700,7 @@
         <v>15</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1663,7 +1721,7 @@
         <v>21</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1684,7 +1742,7 @@
         <v>27</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1705,7 +1763,7 @@
         <v>24</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1726,7 +1784,7 @@
         <v>12</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1747,509 +1805,530 @@
         <v>18</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="n">
-        <f aca="false">'McMaster order'!A18</f>
+        <f aca="false">'McMaster order'!A21</f>
         <v>8</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="n">
-        <f aca="false">'McMaster order'!A19</f>
+        <f aca="false">'McMaster order'!A22</f>
         <v>4</v>
       </c>
       <c r="B15" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>36</v>
-      </c>
       <c r="D15" s="8" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="n">
+        <f aca="false">'McMaster order'!A20</f>
+        <v>4</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="n">
         <f aca="false">'McMaster order'!A17</f>
-        <v>4</v>
-      </c>
-      <c r="B16" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C17" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D17" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E17" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="F17" s="8" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D19&amp;IF($E19="-",""," - "&amp;$E19))</f>
-        <v>1</v>
-      </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>73</v>
-      </c>
+      <c r="A19" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D20&amp;IF($E20="-",""," - "&amp;$E20))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D20&amp;IF($E20="-",""," - "&amp;$E20))</f>
         <v>1</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D21&amp;IF($E21="-",""," - "&amp;$E21))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D21&amp;IF($E21="-",""," - "&amp;$E21))</f>
         <v>1</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D21" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D22&amp;IF($E22="-",""," - "&amp;$E22))</f>
+        <v>1</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E21" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
+      <c r="D22" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D24&amp;IF($E24="-",""," - "&amp;$E24))</f>
-        <v>2</v>
-      </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>82</v>
-      </c>
+      <c r="A24" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D25&amp;IF($E25="-",""," - "&amp;$E25))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D25&amp;IF($E25="-",""," - "&amp;$E25))</f>
         <v>2</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D26&amp;IF($E26="-",""," - "&amp;$E26))</f>
-        <v>1</v>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D26&amp;IF($E26="-",""," - "&amp;$E26))</f>
+        <v>2</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D27&amp;IF($E27="-",""," - "&amp;$E27))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D27&amp;IF($E27="-",""," - "&amp;$E27))</f>
         <v>1</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E27" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F27" s="8" t="s">
         <v>88</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D28&amp;IF($E28="-",""," - "&amp;$E28))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D28&amp;IF($E28="-",""," - "&amp;$E28))</f>
         <v>1</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D29&amp;IF($E29="-",""," - "&amp;$E29))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D29&amp;IF($E29="-",""," - "&amp;$E29))</f>
         <v>1</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D30&amp;IF($E30="-",""," - "&amp;$E30))</f>
+        <v>1</v>
+      </c>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D32&amp;IF($E32="-",""," - "&amp;$E32))</f>
+      <c r="A32" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D33&amp;IF($E33="-",""," - "&amp;$E33))</f>
         <v>2</v>
       </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D35&amp;IF($E35="-",""," - "&amp;$E35))</f>
-        <v>1</v>
-      </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>101</v>
-      </c>
+      <c r="A35" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D36&amp;IF($E36="-",""," - "&amp;$E36))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D36&amp;IF($E36="-",""," - "&amp;$E36))</f>
         <v>1</v>
       </c>
       <c r="B36" s="8"/>
       <c r="C36" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D37&amp;IF($E37="-",""," - "&amp;$E37))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D37&amp;IF($E37="-",""," - "&amp;$E37))</f>
         <v>1</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D38&amp;IF($E38="-",""," - "&amp;$E38))</f>
-        <v>2</v>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D38&amp;IF($E38="-",""," - "&amp;$E38))</f>
+        <v>1</v>
       </c>
       <c r="B38" s="8"/>
       <c r="C38" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D39&amp;IF($E39="-",""," - "&amp;$E39))</f>
-        <v>1</v>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D39&amp;IF($E39="-",""," - "&amp;$E39))</f>
+        <v>2</v>
       </c>
       <c r="B39" s="8"/>
       <c r="C39" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B41" s="6"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
+        <v>118</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D40&amp;IF($E40="-",""," - "&amp;$E40))</f>
+        <v>1</v>
+      </c>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D42&amp;IF($E42="-",""," - "&amp;$E42))</f>
-        <v>1</v>
-      </c>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="F42" s="8" t="s">
-        <v>121</v>
-      </c>
+      <c r="A42" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D43&amp;IF($E43="-",""," - "&amp;$E43))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D43&amp;IF($E43="-",""," - "&amp;$E43))</f>
         <v>1</v>
       </c>
       <c r="B43" s="8"/>
       <c r="C43" s="8" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D44&amp;IF($E44="-",""," - "&amp;$E44))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D44&amp;IF($E44="-",""," - "&amp;$E44))</f>
         <v>1</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="8" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D45&amp;IF($E45="-",""," - "&amp;$E45))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D45&amp;IF($E45="-",""," - "&amp;$E45))</f>
         <v>1</v>
       </c>
       <c r="B45" s="8"/>
       <c r="C45" s="8" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="n">
-        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$40,'By sub-assembly'!$E$2:$E$40,$D46&amp;IF($E46="-",""," - "&amp;$E46))</f>
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D46&amp;IF($E46="-",""," - "&amp;$E46))</f>
         <v>1</v>
       </c>
       <c r="B46" s="8"/>
       <c r="C46" s="8" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="E46" s="8" t="s">
         <v>126</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="10" t="n">
-        <f aca="false">SUM(A4:A47)</f>
-        <v>113</v>
-      </c>
-      <c r="D48" s="10" t="s">
         <v>127</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="n">
+        <f aca="false">SUMIFS('By sub-assembly'!$G$2:$G$41,'By sub-assembly'!$E$2:$E$41,$D47&amp;IF($E47="-",""," - "&amp;$E47))</f>
+        <v>1</v>
+      </c>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10" t="n">
+        <f aca="false">SUM(A4:A48)</f>
+        <v>115</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2268,7 +2347,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="125"/>
@@ -2276,7 +2355,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2284,17 +2363,17 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2302,42 +2381,42 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2345,32 +2424,32 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2378,75 +2457,85 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12"/>
+      <c r="A35" s="12" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12" t="s">
-        <v>159</v>
+      <c r="A37" s="12"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -2465,7 +2554,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
@@ -2478,42 +2567,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="F2" s="13" t="n">
         <v>1</v>
@@ -2525,17 +2614,17 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="F3" s="13" t="n">
         <v>1</v>
@@ -2547,39 +2636,41 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="8" t="s">
+        <v>35</v>
+      </c>
       <c r="E4" s="8" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="8" t="n">
         <f aca="false">C4*F4</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>169</v>
+        <v>62</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="F5" s="13" t="n">
         <v>1</v>
@@ -2591,17 +2682,17 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="8"/>
       <c r="E6" s="8" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="F6" s="13" t="n">
         <v>1</v>
@@ -2613,43 +2704,41 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>50</v>
+        <v>179</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>46</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D7" s="8"/>
       <c r="E7" s="8" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="F7" s="13" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="8" t="n">
         <f aca="false">C7*F7</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="F8" s="13" t="n">
         <v>1</v>
@@ -2661,19 +2750,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="F9" s="13" t="n">
         <v>1</v>
@@ -2688,16 +2777,16 @@
         <v>13</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="F10" s="13" t="n">
         <v>1</v>
@@ -2712,16 +2801,16 @@
         <v>13</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="F11" s="13" t="n">
         <v>1</v>
@@ -2733,113 +2822,113 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="8" t="n">
         <f aca="false">C12*F12</f>
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="8" t="n">
         <f aca="false">C13*F13</f>
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>182</v>
+        <v>50</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="8"/>
+        <v>4</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>48</v>
+      </c>
       <c r="E14" s="8" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>1</v>
       </c>
       <c r="G14" s="8" t="n">
         <f aca="false">C14*F14</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>41</v>
+        <v>192</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>14</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D15" s="8"/>
       <c r="E15" s="8" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="F15" s="13" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="8" t="n">
         <f aca="false">C15*F15</f>
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>8</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>1</v>
@@ -2851,19 +2940,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>8</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F17" s="13" t="n">
         <v>1</v>
@@ -2875,153 +2964,155 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>188</v>
+        <v>47</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="8"/>
+        <v>8</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>45</v>
+      </c>
       <c r="E18" s="8" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="F18" s="13" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="8" t="n">
         <f aca="false">C18*F18</f>
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="8" t="s">
-        <v>14</v>
-      </c>
+      <c r="D19" s="8"/>
       <c r="E19" s="8" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="F19" s="13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G19" s="8" t="n">
         <f aca="false">C19*F19</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G20" s="8" t="n">
         <f aca="false">C20*F20</f>
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="8"/>
+      <c r="D21" s="8" t="s">
+        <v>30</v>
+      </c>
       <c r="E21" s="8" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="F21" s="13" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G21" s="8" t="n">
         <f aca="false">C21*F21</f>
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" s="8" t="n">
         <f aca="false">C22*F22</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="8" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="F23" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23" s="8" t="n">
         <f aca="false">C23*F23</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="F24" s="13" t="n">
         <v>1</v>
@@ -3033,133 +3124,133 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="F25" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" s="8" t="n">
         <f aca="false">C25*F25</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="8" t="s">
-        <v>17</v>
-      </c>
+      <c r="D26" s="8"/>
       <c r="E26" s="8" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="F26" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26" s="8" t="n">
         <f aca="false">C26*F26</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="F27" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G27" s="8" t="n">
         <f aca="false">C27*F27</f>
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>203</v>
-      </c>
       <c r="C28" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="F28" s="13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G28" s="8" t="n">
         <f aca="false">C28*F28</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="B29" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="C29" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="C29" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8" t="s">
-        <v>204</v>
-      </c>
       <c r="F29" s="13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G29" s="8" t="n">
         <f aca="false">C29*F29</f>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="8"/>
       <c r="E30" s="8" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="F30" s="13" t="n">
         <v>1</v>
@@ -3171,19 +3262,17 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>17</v>
-      </c>
+      <c r="D31" s="8"/>
       <c r="E31" s="8" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="F31" s="13" t="n">
         <v>1</v>
@@ -3195,131 +3284,133 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="F32" s="13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G32" s="8" t="n">
         <f aca="false">C32*F32</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="8" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="8"/>
+      <c r="D33" s="8" t="s">
+        <v>23</v>
+      </c>
       <c r="E33" s="8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F33" s="13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G33" s="8" t="n">
         <f aca="false">C33*F33</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D34" s="8" t="s">
-        <v>14</v>
-      </c>
+      <c r="D34" s="8"/>
       <c r="E34" s="8" t="s">
-        <v>186</v>
+        <v>217</v>
       </c>
       <c r="F34" s="13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G34" s="8" t="n">
         <f aca="false">C34*F34</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D35" s="8"/>
+      <c r="D35" s="8" t="s">
+        <v>14</v>
+      </c>
       <c r="E35" s="8" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="F35" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G35" s="8" t="n">
         <f aca="false">C35*F35</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="F36" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" s="8" t="n">
         <f aca="false">C36*F36</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>213</v>
+        <v>176</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D37" s="8"/>
       <c r="E37" s="8" t="s">
-        <v>119</v>
+        <v>220</v>
       </c>
       <c r="F37" s="13" t="n">
         <v>1</v>
@@ -3331,17 +3422,17 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="8" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="8"/>
       <c r="E38" s="8" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F38" s="13" t="n">
         <v>1</v>
@@ -3353,17 +3444,17 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="F39" s="13" t="n">
         <v>1</v>
@@ -3375,17 +3466,17 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D40" s="8"/>
       <c r="E40" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F40" s="13" t="n">
         <v>1</v>
@@ -3396,12 +3487,34 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F41" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="G41" s="10" t="n">
-        <f aca="false">SUM(G2:G40)</f>
-        <v>113</v>
+      <c r="A41" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="C41" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F41" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="8" t="n">
+        <f aca="false">C41*F41</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F42" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="G42" s="10" t="n">
+        <f aca="false">SUM(G2:G41)</f>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>